<commit_message>
pmt and data tab
</commit_message>
<xml_diff>
--- a/New Microsoft Excel Worksheet.xlsx
+++ b/New Microsoft Excel Worksheet.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Cadd Mentor\Student_Class_Code\Siddhi_Vinayak_Files\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52DE87F8-6AF1-4FBA-A9AB-D747E1474C8E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -18,9 +24,116 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="33">
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>Manager</t>
+  </si>
+  <si>
+    <t>SalesMan</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Units</t>
+  </si>
+  <si>
+    <t>Unit_price</t>
+  </si>
+  <si>
+    <t>Sale_amt</t>
+  </si>
+  <si>
+    <t>Payment Type</t>
+  </si>
+  <si>
+    <t>East</t>
+  </si>
+  <si>
+    <t>Martha</t>
+  </si>
+  <si>
+    <t>Alexander</t>
+  </si>
+  <si>
+    <t>Television</t>
+  </si>
+  <si>
+    <t>UPI</t>
+  </si>
+  <si>
+    <t>Central</t>
+  </si>
+  <si>
+    <t>Hermann</t>
+  </si>
+  <si>
+    <t>Shelli</t>
+  </si>
+  <si>
+    <t>Home Theater</t>
+  </si>
+  <si>
+    <t>CASH</t>
+  </si>
+  <si>
+    <t>Indian</t>
+  </si>
+  <si>
+    <t>Luis</t>
+  </si>
+  <si>
+    <t>DEBIT CARD</t>
+  </si>
+  <si>
+    <t>Timothy</t>
+  </si>
+  <si>
+    <t>David</t>
+  </si>
+  <si>
+    <t>Cell Phone</t>
+  </si>
+  <si>
+    <t>NET BANKING</t>
+  </si>
+  <si>
+    <t>West</t>
+  </si>
+  <si>
+    <t>Stephen</t>
+  </si>
+  <si>
+    <t>Steven</t>
+  </si>
+  <si>
+    <t>Douglas</t>
+  </si>
+  <si>
+    <t>Michael</t>
+  </si>
+  <si>
+    <t>Sigal</t>
+  </si>
+  <si>
+    <t>Diana</t>
+  </si>
+  <si>
+    <t>Karen</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,16 +141,36 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -45,12 +178,43 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +494,540 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H64"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="4">
+        <v>95</v>
+      </c>
+      <c r="F2" s="4">
+        <v>1198</v>
+      </c>
+      <c r="G2" s="4">
+        <v>113810</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="6">
+        <v>50</v>
+      </c>
+      <c r="F3" s="6">
+        <v>500</v>
+      </c>
+      <c r="G3" s="6">
+        <v>45000</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="4">
+        <v>36</v>
+      </c>
+      <c r="F4" s="4">
+        <v>1198</v>
+      </c>
+      <c r="G4" s="4">
+        <v>43128</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="6">
+        <v>27</v>
+      </c>
+      <c r="F5" s="6">
+        <v>225</v>
+      </c>
+      <c r="G5" s="6">
+        <v>6075</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="4">
+        <v>56</v>
+      </c>
+      <c r="F6" s="4">
+        <v>1198</v>
+      </c>
+      <c r="G6" s="4">
+        <v>67088</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="6">
+        <v>60</v>
+      </c>
+      <c r="F7" s="6">
+        <v>500</v>
+      </c>
+      <c r="G7" s="6">
+        <v>30000</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="4">
+        <v>75</v>
+      </c>
+      <c r="F8" s="4">
+        <v>1198</v>
+      </c>
+      <c r="G8" s="4">
+        <v>89850</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="6">
+        <v>90</v>
+      </c>
+      <c r="F9" s="6">
+        <v>1198</v>
+      </c>
+      <c r="G9" s="6">
+        <v>107820</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="4">
+        <v>32</v>
+      </c>
+      <c r="F10" s="4">
+        <v>1198</v>
+      </c>
+      <c r="G10" s="4">
+        <v>38336</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="6">
+        <v>60</v>
+      </c>
+      <c r="F11" s="6">
+        <v>500</v>
+      </c>
+      <c r="G11" s="6">
+        <v>30000</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" s="4">
+        <v>90</v>
+      </c>
+      <c r="F12" s="4">
+        <v>1198</v>
+      </c>
+      <c r="G12" s="4">
+        <v>107820</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" s="6">
+        <v>29</v>
+      </c>
+      <c r="F13" s="6">
+        <v>500</v>
+      </c>
+      <c r="G13" s="6">
+        <v>14500</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E14" s="4">
+        <v>81</v>
+      </c>
+      <c r="F14" s="4">
+        <v>500</v>
+      </c>
+      <c r="G14" s="4">
+        <v>40500</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" s="6">
+        <v>35</v>
+      </c>
+      <c r="F15" s="6">
+        <v>1198</v>
+      </c>
+      <c r="G15" s="6">
+        <v>41930</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H22" s="1"/>
+    </row>
+    <row r="23" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H23" s="1"/>
+    </row>
+    <row r="24" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H24" s="1"/>
+    </row>
+    <row r="25" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H25" s="1"/>
+    </row>
+    <row r="26" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H26" s="1"/>
+    </row>
+    <row r="27" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H27" s="1"/>
+    </row>
+    <row r="28" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H28" s="1"/>
+    </row>
+    <row r="29" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H29" s="1"/>
+    </row>
+    <row r="30" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H30" s="1"/>
+    </row>
+    <row r="31" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H31" s="1"/>
+    </row>
+    <row r="32" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H32" s="1"/>
+    </row>
+    <row r="33" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H33" s="1"/>
+    </row>
+    <row r="34" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H34" s="1"/>
+    </row>
+    <row r="35" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H35" s="1"/>
+    </row>
+    <row r="36" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H36" s="1"/>
+    </row>
+    <row r="37" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H37" s="1"/>
+    </row>
+    <row r="38" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H38" s="1"/>
+    </row>
+    <row r="39" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H39" s="1"/>
+    </row>
+    <row r="40" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H40" s="1"/>
+    </row>
+    <row r="41" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H41" s="1"/>
+    </row>
+    <row r="42" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H42" s="1"/>
+    </row>
+    <row r="43" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H43" s="1"/>
+    </row>
+    <row r="44" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H44" s="1"/>
+    </row>
+    <row r="45" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H45" s="1"/>
+    </row>
+    <row r="46" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H46" s="1"/>
+    </row>
+    <row r="47" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H47" s="1"/>
+    </row>
+    <row r="48" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H48" s="1"/>
+    </row>
+    <row r="49" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H49" s="1"/>
+    </row>
+    <row r="50" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H50" s="1"/>
+    </row>
+    <row r="51" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H51" s="1"/>
+    </row>
+    <row r="52" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H52" s="1"/>
+    </row>
+    <row r="53" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H53" s="1"/>
+    </row>
+    <row r="54" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H54" s="1"/>
+    </row>
+    <row r="55" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H55" s="1"/>
+    </row>
+    <row r="56" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H56" s="1"/>
+    </row>
+    <row r="57" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H57" s="1"/>
+    </row>
+    <row r="58" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H58" s="1"/>
+    </row>
+    <row r="59" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H59" s="1"/>
+    </row>
+    <row r="60" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H60" s="1"/>
+    </row>
+    <row r="61" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H61" s="1"/>
+    </row>
+    <row r="62" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H62" s="1"/>
+    </row>
+    <row r="63" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H63" s="1"/>
+    </row>
+    <row r="64" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H64" s="1"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>